<commit_message>
k and p values
</commit_message>
<xml_diff>
--- a/Comparison Table of k and p Values.xlsx
+++ b/Comparison Table of k and p Values.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/Assignment-1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="20" documentId="8_{F5548F79-425C-4B76-B71C-57BD59B12E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D212EABC-19FF-4AD6-B916-EDDBB28A8C09}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="8_{F5548F79-425C-4B76-B71C-57BD59B12E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CF0F48B-2FDD-4998-A6AA-A58429021401}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D244108E-BDF8-4038-A556-2A9E06F46F59}"/>
   </bookViews>
@@ -160,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -169,9 +169,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -535,48 +532,48 @@
       <c r="E1" s="1"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="8" t="s">
+      <c r="C2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="6" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="3">
         <v>0.5</v>
       </c>
       <c r="C3" s="3">
-        <v>0.61709999999999998</v>
-      </c>
-      <c r="D3" s="5">
+        <v>0.49730000000000002</v>
+      </c>
+      <c r="D3" s="4">
         <v>1</v>
       </c>
-      <c r="E3" s="4"/>
+      <c r="E3" s="4">
+        <v>0.99960000000000004</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3">
-        <v>0.98089999999999999</v>
-      </c>
+      <c r="B4" s="3"/>
       <c r="C4" s="3">
         <v>3.7699999999999997E-2</v>
       </c>
-      <c r="D4" s="5">
+      <c r="D4" s="4">
         <v>2</v>
       </c>
       <c r="E4" s="4">
@@ -584,7 +581,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -593,10 +590,10 @@
       <c r="C5" s="3">
         <v>0.1522</v>
       </c>
-      <c r="D5" s="5">
+      <c r="D5" s="4">
         <v>1.6</v>
       </c>
-      <c r="E5" s="5">
+      <c r="E5" s="4">
         <v>1.6215999999999999</v>
       </c>
     </row>

</xml_diff>

<commit_message>
calculate k for newtons
</commit_message>
<xml_diff>
--- a/Comparison Table of k and p Values.xlsx
+++ b/Comparison Table of k and p Values.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/mepstein_olin_edu/Documents/Desktop/Applied Math/Assignment-1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://olincollege-my.sharepoint.com/personal/kyue_olin_edu/Documents/Documents/MATLAB/Numerical Methods/Assignment-1/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="8_{F5548F79-425C-4B76-B71C-57BD59B12E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7CF0F48B-2FDD-4998-A6AA-A58429021401}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{F5548F79-425C-4B76-B71C-57BD59B12E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C2EE308-B5DF-418E-A7BB-A41033188973}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{D244108E-BDF8-4038-A556-2A9E06F46F59}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{D244108E-BDF8-4038-A556-2A9E06F46F59}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
   <si>
     <t>Comparison Table of k and p Values</t>
   </si>
@@ -69,6 +69,9 @@
   </si>
   <si>
     <t>N/A</t>
+  </si>
+  <si>
+    <t>Fzero Method</t>
   </si>
 </sst>
 </file>
@@ -162,9 +165,6 @@
   </cellStyleXfs>
   <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -178,6 +178,9 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -193,6 +196,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -523,82 +530,101 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="8" t="s">
+      <c r="A2" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="7" t="s">
+      <c r="B2" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="7" t="s">
+      <c r="C2" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="5" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>0.5</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="2">
         <v>0.49730000000000002</v>
       </c>
-      <c r="D3" s="4">
+      <c r="D3" s="3">
         <v>1</v>
       </c>
-      <c r="E3" s="4">
+      <c r="E3" s="3">
         <v>0.99960000000000004</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3">
-        <v>3.7699999999999997E-2</v>
-      </c>
-      <c r="D4" s="4">
+      <c r="B4" s="2">
+        <v>3.73E-2</v>
+      </c>
+      <c r="C4" s="2">
+        <v>3.7600000000000001E-2</v>
+      </c>
+      <c r="D4" s="3">
         <v>2</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4" s="3">
         <v>1.9995000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="2">
         <v>0.1522</v>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="3">
         <v>1.6</v>
       </c>
-      <c r="E5" s="4">
+      <c r="E5" s="3">
         <v>1.6215999999999999</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2">
+        <v>0.12429999999999999</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1.6648000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="C8" s="2"/>
+      <c r="C8" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>